<commit_message>
create data file as example for 2019 values
</commit_message>
<xml_diff>
--- a/01_data/02_output_data/02_unidirectional_results/01_paper_IAEE/02_prepared_results/emission_differences.xlsx
+++ b/01_data/02_output_data/02_unidirectional_results/01_paper_IAEE/02_prepared_results/emission_differences.xlsx
@@ -1,22 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\02_output_data\02_unidirectional_results\01_paper_IAEE\02_prepared_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6456E1F-E9CB-4A67-8E6B-0054B3C91551}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{810A1E09-6261-441C-BE6B-2D80CFB66BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Emissions_Europe" sheetId="1" r:id="rId1"/>
     <sheet name="Emissions_EU" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -115,11 +128,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -423,16 +439,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.7265625" customWidth="1"/>
-    <col min="2" max="2" width="22.1796875" customWidth="1"/>
-    <col min="3" max="3" width="23.1796875" customWidth="1"/>
-    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="2" max="2" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -446,130 +463,195 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="2">
-        <v>200224130.88433269</v>
-      </c>
-      <c r="C2" s="2">
+      <c r="B2" s="3">
+        <v>204453208.3558054</v>
+      </c>
+      <c r="C2" s="3">
         <v>11179725.52237861</v>
       </c>
-      <c r="D2" s="2">
-        <v>211403856.4067114</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D2" s="3">
+        <v>215632933.87818399</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="2">
-        <v>179994391.54406461</v>
-      </c>
-      <c r="C3" s="2">
+      <c r="B3" s="3">
+        <v>185554176.49482459</v>
+      </c>
+      <c r="C3" s="3">
         <v>10383166.675329819</v>
       </c>
-      <c r="D3" s="2">
-        <v>190377558.21939439</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D3" s="3">
+        <v>195937343.17015439</v>
+      </c>
+      <c r="G3">
+        <f>D3/$D$2</f>
+        <v>0.90866149083165515</v>
+      </c>
+      <c r="H3">
+        <f>1-G3</f>
+        <v>9.133850916834485E-2</v>
+      </c>
+      <c r="J3" s="5"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="2">
-        <v>179884321.3980023</v>
-      </c>
-      <c r="C4" s="2">
+      <c r="B4" s="3">
+        <v>185496745.98499781</v>
+      </c>
+      <c r="C4" s="3">
         <v>10626696.013548739</v>
       </c>
-      <c r="D4" s="2">
-        <v>190511017.411551</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D4" s="3">
+        <v>196123441.99854651</v>
+      </c>
+      <c r="G4" s="4">
+        <f>D4/$D$2</f>
+        <v>0.90952452610667145</v>
+      </c>
+      <c r="H4" s="4">
+        <f>1-G4</f>
+        <v>9.0475473893328551E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="2">
-        <v>179990414.9475081</v>
-      </c>
-      <c r="C5" s="2">
+      <c r="B5" s="3">
+        <v>185550199.89826819</v>
+      </c>
+      <c r="C5" s="3">
         <v>10383166.675329819</v>
       </c>
-      <c r="D5" s="2">
-        <v>190373581.62283799</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D5" s="3">
+        <v>195933366.573598</v>
+      </c>
+      <c r="G5" s="4">
+        <f>D5/$D$2</f>
+        <v>0.90864304932327855</v>
+      </c>
+      <c r="H5" s="4">
+        <f>1-G5</f>
+        <v>9.1356950676721449E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="2">
-        <v>180016621.79081789</v>
-      </c>
-      <c r="C6" s="2">
+      <c r="B6" s="3">
+        <v>185638254.0159592</v>
+      </c>
+      <c r="C6" s="3">
         <v>9895360.668074714</v>
       </c>
-      <c r="D6" s="2">
-        <v>189911982.4588927</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D6" s="3">
+        <v>195533614.68403399</v>
+      </c>
+      <c r="G6" s="4">
+        <f>D6/$D$2</f>
+        <v>0.90678919572877226</v>
+      </c>
+      <c r="H6" s="4">
+        <f>1-G6</f>
+        <v>9.3210804271227743E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="2">
-        <v>152346911.43175361</v>
-      </c>
-      <c r="C7" s="2">
+      <c r="B7" s="3">
+        <v>157885746.4130826</v>
+      </c>
+      <c r="C7" s="3">
         <v>10237072.6112445</v>
       </c>
-      <c r="D7" s="2">
-        <v>162583984.04299799</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D7" s="3">
+        <v>168122819.0243271</v>
+      </c>
+      <c r="G7" s="4">
+        <f>D7/$D$2</f>
+        <v>0.77967134240868585</v>
+      </c>
+      <c r="H7">
+        <f>1-G7</f>
+        <v>0.22032865759131415</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="2">
-        <v>163084040.62762421</v>
-      </c>
-      <c r="C8" s="2">
+      <c r="B8" s="3">
+        <v>168653467.05633211</v>
+      </c>
+      <c r="C8" s="3">
         <v>10226650.072517119</v>
       </c>
-      <c r="D8" s="2">
-        <v>173310690.70014131</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D8" s="3">
+        <v>178880117.12884921</v>
+      </c>
+      <c r="G8" s="4">
+        <f>D8/$D$2</f>
+        <v>0.82955842556917914</v>
+      </c>
+      <c r="H8" s="4">
+        <f>1-G8</f>
+        <v>0.17044157443082086</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="2">
-        <v>94644166.688246429</v>
-      </c>
-      <c r="C9" s="2">
+      <c r="B9" s="3">
+        <v>100414486.3201661</v>
+      </c>
+      <c r="C9" s="3">
         <v>5155714.0202392116</v>
       </c>
-      <c r="D9" s="2">
-        <v>99799880.708485633</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D9" s="3">
+        <v>105570200.3404053</v>
+      </c>
+      <c r="G9" s="4">
+        <f>D9/$D$2</f>
+        <v>0.48958291501076706</v>
+      </c>
+      <c r="H9" s="4">
+        <f>1-G9</f>
+        <v>0.51041708498923288</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="2">
-        <v>151818137.9500474</v>
-      </c>
-      <c r="C10" s="2">
+      <c r="B10" s="3">
+        <v>157745173.08999321</v>
+      </c>
+      <c r="C10" s="3">
         <v>8920010.1605223659</v>
       </c>
-      <c r="D10" s="2">
-        <v>160738148.11056969</v>
+      <c r="D10" s="3">
+        <v>166665183.25051561</v>
+      </c>
+      <c r="G10" s="4">
+        <f>D10/$D$2</f>
+        <v>0.7729115411687002</v>
+      </c>
+      <c r="H10" s="4">
+        <f>1-G10</f>
+        <v>0.2270884588312998</v>
       </c>
     </row>
   </sheetData>
@@ -579,16 +661,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.54296875" customWidth="1"/>
-    <col min="2" max="2" width="21.6328125" customWidth="1"/>
-    <col min="3" max="3" width="23.90625" customWidth="1"/>
-    <col min="4" max="4" width="20.453125" customWidth="1"/>
+    <col min="2" max="2" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -602,131 +683,140 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B2" s="2">
-        <v>143035009.3409034</v>
+        <v>147264086.81237599</v>
       </c>
       <c r="C2" s="2">
         <v>5811815.7394667082</v>
       </c>
       <c r="D2" s="2">
-        <v>148846825.0803701</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+        <v>153075902.55184269</v>
+      </c>
+      <c r="E2" s="2"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B3" s="2">
-        <v>147134073.67407581</v>
+        <v>152693858.62483579</v>
       </c>
       <c r="C3" s="2">
         <v>4605256.903954668</v>
       </c>
       <c r="D3" s="2">
-        <v>151739330.57803041</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+        <v>157299115.5287905</v>
+      </c>
+      <c r="E3" s="2"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="2">
-        <v>140389751.05994391</v>
+        <v>146002175.6469394</v>
       </c>
       <c r="C4" s="2">
         <v>4848623.6498271329</v>
       </c>
       <c r="D4" s="2">
-        <v>145238374.70977101</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+        <v>150850799.29676661</v>
+      </c>
+      <c r="E4" s="2"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B5" s="2">
-        <v>147099685.13339141</v>
+        <v>152659470.08415139</v>
       </c>
       <c r="C5" s="2">
         <v>4605256.903954668</v>
       </c>
       <c r="D5" s="2">
-        <v>151704942.03734609</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+        <v>157264726.9881061</v>
+      </c>
+      <c r="E5" s="2"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B6" s="2">
-        <v>152074545.14187989</v>
+        <v>157536419.65140399</v>
       </c>
       <c r="C6" s="2">
         <v>4483440.6559147602</v>
       </c>
       <c r="D6" s="2">
-        <v>156557985.7977947</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+        <v>162019860.30731881</v>
+      </c>
+      <c r="E6" s="2"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B7" s="2">
-        <v>126386110.2648232</v>
+        <v>131924945.2461523</v>
       </c>
       <c r="C7" s="2">
         <v>4468687.0231602956</v>
       </c>
       <c r="D7" s="2">
-        <v>130854797.28798351</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+        <v>136393632.2693125</v>
+      </c>
+      <c r="E7" s="2"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B8" s="2">
-        <v>141071131.29630879</v>
+        <v>146640557.72501671</v>
       </c>
       <c r="C8" s="2">
         <v>4612862.7479998441</v>
       </c>
       <c r="D8" s="2">
-        <v>145683994.04430869</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+        <v>151253420.47301659</v>
+      </c>
+      <c r="E8" s="2"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B9" s="2">
-        <v>78297727.204894096</v>
+        <v>83762047.463099182</v>
       </c>
       <c r="C9" s="2">
         <v>1139802.8320675341</v>
       </c>
       <c r="D9" s="2">
-        <v>79437530.036961645</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+        <v>84901850.295166731</v>
+      </c>
+      <c r="E9" s="2"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B10" s="2">
-        <v>124042398.08937269</v>
+        <v>129969433.2293186</v>
       </c>
       <c r="C10" s="2">
         <v>3757180.883541625</v>
       </c>
       <c r="D10" s="2">
-        <v>127799578.97291429</v>
-      </c>
+        <v>133726614.1128602</v>
+      </c>
+      <c r="E10" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>